<commit_message>
v2.1.1: reportes por caja, fechas de entrega, IEPS/IVA, plantillas editables y precios masivos por cliente
</commit_message>
<xml_diff>
--- a/sku-servidor/public/layout-clientes.xlsx
+++ b/sku-servidor/public/layout-clientes.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLIENTES" sheetId="1" r:id="R6789f55d7ab14893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EJEMPLOS" sheetId="2" r:id="R2f1d857ac8104722"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLIENTES" sheetId="1" r:id="Rb8b1fad47cac45bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EJEMPLOS" sheetId="2" r:id="R39366b97f70f41c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2560,7 +2560,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re02a84680fb54294"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde0bc5b58d314d7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>